<commit_message>
fix: PlayerController null 체크 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/PreLoadAsset.xlsx
+++ b/JsonConverter/ExcelFiles/PreLoadAsset.xlsx
@@ -1,15 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="enqOkH1Z/tfQ3WIfr7wm+HPEzSLVVhkZawHcM088EJg="/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -459,41 +470,190 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="23">
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Malgun Gothic"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Malgun Gothic"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Malgun Gothic"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color theme="1"/>
-      <name val="Malgun Gothic"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -501,68 +661,736 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
-    <border/>
+  <borders count="9">
     <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFB2B2B2"/>
       </right>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color rgb="FFB2B2B2"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+  <cellXfs count="11">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="49">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="17">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <left style="thin">
+          <color theme="4"/>
+        </left>
+        <right style="thin">
+          <color theme="4"/>
+        </right>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+        <horizontal style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
+  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    </tableStyle>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -752,23 +1580,23 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C1000"/>
+  <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1" outlineLevelCol="2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="52.14"/>
-    <col customWidth="1" min="2" max="2" width="35.14"/>
-    <col customWidth="1" min="3" max="3" width="31.43"/>
-    <col customWidth="1" min="4" max="26" width="9.0"/>
+    <col min="1" max="1" width="52.1388888888889" customWidth="1"/>
+    <col min="2" max="2" width="35.1388888888889" customWidth="1"/>
+    <col min="3" max="3" width="31.4259259259259" customWidth="1"/>
+    <col min="4" max="26" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1">
+    <row r="1" ht="17.25" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -779,7 +1607,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" ht="17.25" customHeight="1">
+    <row r="2" ht="17.25" customHeight="1" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -790,7 +1618,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="17.25" customHeight="1">
+    <row r="3" ht="17.25" customHeight="1" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -801,7 +1629,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="17.25" customHeight="1">
+    <row r="4" ht="17.25" customHeight="1" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -809,7 +1637,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="17.25" customHeight="1">
+    <row r="5" ht="17.25" customHeight="1" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -817,7 +1645,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" ht="17.25" customHeight="1">
+    <row r="6" ht="17.25" customHeight="1" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -825,7 +1653,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" ht="17.25" customHeight="1">
+    <row r="7" ht="17.25" customHeight="1" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -833,7 +1661,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" ht="17.25" customHeight="1">
+    <row r="8" ht="17.25" customHeight="1" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -841,7 +1669,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" ht="17.25" customHeight="1">
+    <row r="9" ht="17.25" customHeight="1" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -849,7 +1677,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" ht="17.25" customHeight="1">
+    <row r="10" ht="17.25" customHeight="1" spans="1:3">
       <c r="A10" s="1" t="s">
         <v>19</v>
       </c>
@@ -857,7 +1685,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" ht="17.25" customHeight="1">
+    <row r="11" ht="17.25" customHeight="1" spans="1:3">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -865,7 +1693,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" ht="17.25" customHeight="1">
+    <row r="12" ht="17.25" customHeight="1" spans="1:3">
       <c r="A12" s="1" t="s">
         <v>23</v>
       </c>
@@ -873,7 +1701,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" ht="17.25" customHeight="1">
+    <row r="13" ht="17.25" customHeight="1" spans="1:3">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
@@ -881,7 +1709,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" ht="17.25" customHeight="1">
+    <row r="14" ht="17.25" customHeight="1" spans="1:3">
       <c r="A14" s="1" t="s">
         <v>27</v>
       </c>
@@ -889,7 +1717,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" ht="17.25" customHeight="1">
+    <row r="15" ht="17.25" customHeight="1" spans="1:3">
       <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
@@ -897,7 +1725,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" ht="17.25" customHeight="1">
+    <row r="16" ht="17.25" customHeight="1" spans="1:3">
       <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
@@ -905,7 +1733,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" ht="17.25" customHeight="1">
+    <row r="17" ht="17.25" customHeight="1" spans="1:2">
       <c r="A17" s="1" t="s">
         <v>33</v>
       </c>
@@ -913,7 +1741,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" ht="17.25" customHeight="1">
+    <row r="18" ht="17.25" customHeight="1" spans="1:2">
       <c r="A18" s="1" t="s">
         <v>35</v>
       </c>
@@ -921,7 +1749,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" ht="17.25" customHeight="1">
+    <row r="19" ht="17.25" customHeight="1" spans="1:2">
       <c r="A19" s="1" t="s">
         <v>37</v>
       </c>
@@ -929,7 +1757,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" ht="17.25" customHeight="1">
+    <row r="20" ht="17.25" customHeight="1" spans="1:2">
       <c r="A20" s="1" t="s">
         <v>39</v>
       </c>
@@ -937,7 +1765,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" ht="17.25" customHeight="1">
+    <row r="21" ht="17.25" customHeight="1" spans="1:2">
       <c r="A21" s="1" t="s">
         <v>41</v>
       </c>
@@ -945,7 +1773,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" ht="17.25" customHeight="1">
+    <row r="22" ht="17.25" customHeight="1" spans="1:2">
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
@@ -953,7 +1781,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" ht="17.25" customHeight="1">
+    <row r="23" ht="17.25" customHeight="1" spans="1:2">
       <c r="A23" s="1" t="s">
         <v>45</v>
       </c>
@@ -961,7 +1789,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="24" ht="17.25" customHeight="1">
+    <row r="24" ht="17.25" customHeight="1" spans="1:2">
       <c r="A24" s="1" t="s">
         <v>47</v>
       </c>
@@ -969,7 +1797,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="25" ht="17.25" customHeight="1">
+    <row r="25" ht="17.25" customHeight="1" spans="1:2">
       <c r="A25" s="1" t="s">
         <v>49</v>
       </c>
@@ -977,7 +1805,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" ht="17.25" customHeight="1">
+    <row r="26" ht="17.25" customHeight="1" spans="1:2">
       <c r="A26" s="1" t="s">
         <v>51</v>
       </c>
@@ -985,7 +1813,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" ht="17.25" customHeight="1">
+    <row r="27" ht="17.25" customHeight="1" spans="1:2">
       <c r="A27" s="1" t="s">
         <v>53</v>
       </c>
@@ -993,7 +1821,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="28" ht="17.25" customHeight="1">
+    <row r="28" ht="17.25" customHeight="1" spans="1:2">
       <c r="A28" s="1" t="s">
         <v>55</v>
       </c>
@@ -1001,7 +1829,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" ht="17.25" customHeight="1">
+    <row r="29" ht="17.25" customHeight="1" spans="1:2">
       <c r="A29" s="1" t="s">
         <v>57</v>
       </c>
@@ -1009,7 +1837,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" ht="17.25" customHeight="1">
+    <row r="30" ht="17.25" customHeight="1" spans="1:2">
       <c r="A30" s="1" t="s">
         <v>59</v>
       </c>
@@ -1017,7 +1845,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="31" ht="17.25" customHeight="1">
+    <row r="31" ht="17.25" customHeight="1" spans="1:2">
       <c r="A31" s="1" t="s">
         <v>61</v>
       </c>
@@ -1025,7 +1853,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="32" ht="17.25" customHeight="1">
+    <row r="32" ht="17.25" customHeight="1" spans="1:2">
       <c r="A32" s="1" t="s">
         <v>63</v>
       </c>
@@ -1033,7 +1861,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" ht="17.25" customHeight="1">
+    <row r="33" ht="17.25" customHeight="1" spans="1:2">
       <c r="A33" s="1" t="s">
         <v>65</v>
       </c>
@@ -1041,7 +1869,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="34" ht="17.25" customHeight="1">
+    <row r="34" ht="17.25" customHeight="1" spans="1:2">
       <c r="A34" s="1" t="s">
         <v>67</v>
       </c>
@@ -1049,7 +1877,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="35" ht="17.25" customHeight="1">
+    <row r="35" ht="17.25" customHeight="1" spans="1:2">
       <c r="A35" s="1" t="s">
         <v>69</v>
       </c>
@@ -1057,7 +1885,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="36" ht="17.25" customHeight="1">
+    <row r="36" ht="17.25" customHeight="1" spans="1:2">
       <c r="A36" s="1" t="s">
         <v>71</v>
       </c>
@@ -1065,7 +1893,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="37" ht="17.25" customHeight="1">
+    <row r="37" ht="17.25" customHeight="1" spans="1:2">
       <c r="A37" s="1" t="s">
         <v>73</v>
       </c>
@@ -1073,7 +1901,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" ht="17.25" customHeight="1">
+    <row r="38" ht="17.25" customHeight="1" spans="1:2">
       <c r="A38" s="1" t="s">
         <v>75</v>
       </c>
@@ -1081,7 +1909,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="39" ht="17.25" customHeight="1">
+    <row r="39" ht="17.25" customHeight="1" spans="1:2">
       <c r="A39" s="1" t="s">
         <v>77</v>
       </c>
@@ -1089,7 +1917,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="40" ht="17.25" customHeight="1">
+    <row r="40" ht="17.25" customHeight="1" spans="1:2">
       <c r="A40" s="1" t="s">
         <v>79</v>
       </c>
@@ -1097,7 +1925,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41" ht="17.25" customHeight="1">
+    <row r="41" ht="17.25" customHeight="1" spans="1:2">
       <c r="A41" s="1" t="s">
         <v>81</v>
       </c>
@@ -1105,7 +1933,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="42" ht="17.25" customHeight="1">
+    <row r="42" ht="17.25" customHeight="1" spans="1:2">
       <c r="A42" s="1" t="s">
         <v>83</v>
       </c>
@@ -1113,7 +1941,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="43" ht="17.25" customHeight="1">
+    <row r="43" ht="17.25" customHeight="1" spans="1:2">
       <c r="A43" s="1" t="s">
         <v>85</v>
       </c>
@@ -1121,7 +1949,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="44" ht="17.25" customHeight="1">
+    <row r="44" ht="17.25" customHeight="1" spans="1:2">
       <c r="A44" s="1" t="s">
         <v>87</v>
       </c>
@@ -1129,7 +1957,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="45" ht="17.25" customHeight="1">
+    <row r="45" ht="17.25" customHeight="1" spans="1:2">
       <c r="A45" s="1" t="s">
         <v>89</v>
       </c>
@@ -1137,7 +1965,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="46" ht="17.25" customHeight="1">
+    <row r="46" ht="17.25" customHeight="1" spans="1:2">
       <c r="A46" s="1" t="s">
         <v>91</v>
       </c>
@@ -1145,7 +1973,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="47" ht="17.25" customHeight="1">
+    <row r="47" ht="17.25" customHeight="1" spans="1:2">
       <c r="A47" s="2" t="s">
         <v>93</v>
       </c>
@@ -1153,7 +1981,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="48" ht="17.25" customHeight="1">
+    <row r="48" ht="17.25" customHeight="1" spans="1:2">
       <c r="A48" s="2" t="s">
         <v>95</v>
       </c>
@@ -1161,109 +1989,109 @@
         <v>96</v>
       </c>
     </row>
-    <row r="49" ht="17.25" customHeight="1">
-      <c r="A49" s="2" t="s">
+    <row r="49" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A49" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="5" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="50" ht="17.25" customHeight="1">
-      <c r="A50" s="2" t="s">
+    <row r="50" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A50" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="4" t="s">
         <v>100</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="51" ht="17.25" customHeight="1">
-      <c r="A51" s="2" t="s">
+    <row r="51" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A51" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" s="6" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="52" ht="17.25" customHeight="1">
-      <c r="A52" s="2" t="s">
+    <row r="52" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A52" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="6" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="53" ht="17.25" customHeight="1">
-      <c r="A53" s="2" t="s">
+    <row r="53" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A53" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B53" s="4" t="s">
+      <c r="B53" s="6" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="54" ht="17.25" customHeight="1">
-      <c r="A54" s="2" t="s">
+    <row r="54" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A54" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B54" s="6" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="55" ht="17.25" customHeight="1">
-      <c r="A55" s="2" t="s">
+    <row r="55" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A55" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="56" ht="17.25" customHeight="1">
-      <c r="A56" s="2" t="s">
+    <row r="56" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A56" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="6" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="57" ht="17.25" customHeight="1">
-      <c r="A57" s="2" t="s">
+    <row r="57" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A57" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B57" s="5" t="s">
+      <c r="B57" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="58" ht="17.25" customHeight="1">
-      <c r="A58" s="2" t="s">
+    <row r="58" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A58" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B58" s="6" t="s">
+      <c r="B58" s="8" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="59" ht="17.25" customHeight="1">
-      <c r="A59" s="2" t="s">
+    <row r="59" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A59" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="B59" s="6" t="s">
+      <c r="B59" s="8" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="60" ht="17.25" customHeight="1">
-      <c r="A60" s="6" t="s">
+    <row r="60" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A60" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B60" s="6" t="s">
+      <c r="B60" s="9" t="s">
         <v>121</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="61" ht="17.25" customHeight="1">
+    <row r="61" ht="17.25" customHeight="1" spans="1:3">
       <c r="A61" s="2" t="s">
         <v>122</v>
       </c>
@@ -1271,91 +2099,91 @@
         <v>123</v>
       </c>
     </row>
-    <row r="62" ht="17.25" customHeight="1">
-      <c r="A62" s="7" t="s">
+    <row r="62" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A62" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B62" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="63" ht="17.25" customHeight="1">
-      <c r="A63" s="7" t="s">
+    <row r="63" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A63" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="B63" s="8" t="s">
+      <c r="B63" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="64" ht="17.25" customHeight="1">
-      <c r="A64" s="7" t="s">
+    <row r="64" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A64" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="B64" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="65" ht="17.25" customHeight="1">
-      <c r="A65" s="7" t="s">
+    <row r="65" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A65" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="B65" s="8" t="s">
+      <c r="B65" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="66" ht="17.25" customHeight="1">
-      <c r="A66" s="7" t="s">
+    <row r="66" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A66" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="B66" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="67" ht="17.25" customHeight="1">
-      <c r="A67" s="7" t="s">
+    <row r="67" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A67" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="B67" s="8" t="s">
+      <c r="B67" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="68" ht="17.25" customHeight="1">
-      <c r="A68" s="7" t="s">
+    <row r="68" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A68" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="B68" s="8" t="s">
+      <c r="B68" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="69" ht="17.25" customHeight="1">
-      <c r="A69" s="7" t="s">
+    <row r="69" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A69" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="B69" s="8" t="s">
+      <c r="B69" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="70" ht="17.25" customHeight="1">
-      <c r="A70" s="7" t="s">
+    <row r="70" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A70" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B70" s="8" t="s">
+      <c r="B70" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="71" ht="17.25" customHeight="1">
-      <c r="A71" s="8" t="s">
+    <row r="71" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A71" t="s">
         <v>142</v>
       </c>
-      <c r="B71" s="8" t="s">
+      <c r="B71" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="72" ht="17.25" customHeight="1">
-      <c r="A72" s="8" t="s">
+    <row r="72" ht="17.25" customHeight="1" spans="1:2">
+      <c r="A72" t="s">
         <v>144</v>
       </c>
-      <c r="B72" s="8" t="s">
+      <c r="B72" t="s">
         <v>145</v>
       </c>
     </row>
@@ -2288,9 +3116,8 @@
     <row r="999" ht="17.25" customHeight="1"/>
     <row r="1000" ht="17.25" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="1" orientation="landscape"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: 함정 소환을 위한 BaseTrap 구현, 함정 소환, CeilingProvider 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/PreLoadAsset.xlsx
+++ b/JsonConverter/ExcelFiles/PreLoadAsset.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="248">
   <si>
     <t>미리 로드할 어드레서블 테이블</t>
   </si>
@@ -730,6 +730,36 @@
   </si>
   <si>
     <t>ItemObject</t>
+  </si>
+  <si>
+    <t>PreLoadAsset_GameObject_Turret</t>
+  </si>
+  <si>
+    <t>TurretTrap</t>
+  </si>
+  <si>
+    <t>PreLoadAsset_GameObject_Turret_Bullet</t>
+  </si>
+  <si>
+    <t>Turret_Bullet</t>
+  </si>
+  <si>
+    <t>PreLoadAsset_GameObject_StonTrap</t>
+  </si>
+  <si>
+    <t>StonTrap</t>
+  </si>
+  <si>
+    <t>PreLoadAsset_GameObject_WebTrap</t>
+  </si>
+  <si>
+    <t>WebTrap</t>
+  </si>
+  <si>
+    <t>PreLoadAsset_GameObject_BaseTrap</t>
+  </si>
+  <si>
+    <t>BaseTrap</t>
   </si>
 </sst>
 </file>
@@ -2113,11 +2143,46 @@
         <v>237</v>
       </c>
     </row>
-    <row r="119" ht="17.25" customHeight="1"/>
-    <row r="120" ht="17.25" customHeight="1"/>
-    <row r="121" ht="17.25" customHeight="1"/>
-    <row r="122" ht="17.25" customHeight="1"/>
-    <row r="123" ht="17.25" customHeight="1"/>
+    <row r="119" ht="17.25" customHeight="1">
+      <c r="A119" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="B119" s="10" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="120" ht="17.25" customHeight="1">
+      <c r="A120" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B120" s="10" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="121" ht="17.25" customHeight="1">
+      <c r="A121" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="B121" s="10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="122" ht="17.25" customHeight="1">
+      <c r="A122" s="10" t="s">
+        <v>244</v>
+      </c>
+      <c r="B122" s="10" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="123" ht="17.25" customHeight="1">
+      <c r="A123" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="B123" s="10" t="s">
+        <v>247</v>
+      </c>
+    </row>
     <row r="124" ht="17.25" customHeight="1"/>
     <row r="125" ht="17.25" customHeight="1"/>
     <row r="126" ht="17.25" customHeight="1"/>

</xml_diff>

<commit_message>
fix: 플레이어 cinemachinecamera Priority값 수정, 게임 종료 조건 (체포) 체크
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/PreLoadAsset.xlsx
+++ b/JsonConverter/ExcelFiles/PreLoadAsset.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="256">
   <si>
     <t>미리 로드할 어드레서블 테이블</t>
   </si>
@@ -777,6 +777,12 @@
   </si>
   <si>
     <t>MushroomTrap</t>
+  </si>
+  <si>
+    <t>PreLoadAsset_Mesh_MushroomTrap</t>
+  </si>
+  <si>
+    <t>Mashroom_1</t>
   </si>
   <si>
     <t>PreLoadAsset_Material_Color_1</t>
@@ -1969,7 +1975,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C999"/>
+  <dimension ref="A1:C1000"/>
   <sheetFormatPr defaultColWidth="14.4259259259259" defaultRowHeight="15" customHeight="1" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="52.1388888888889" customWidth="1"/>
@@ -3054,6 +3060,9 @@
       <c r="B125" t="s">
         <v>251</v>
       </c>
+      <c r="C125" t="s">
+        <v>103</v>
+      </c>
     </row>
     <row r="126" ht="17.25" customHeight="1" spans="1:3">
       <c r="A126" t="s">
@@ -3063,7 +3072,14 @@
         <v>253</v>
       </c>
     </row>
-    <row r="127" ht="17.25" customHeight="1"/>
+    <row r="127" ht="17.25" customHeight="1" spans="1:3">
+      <c r="A127" t="s">
+        <v>254</v>
+      </c>
+      <c r="B127" t="s">
+        <v>255</v>
+      </c>
+    </row>
     <row r="128" ht="17.25" customHeight="1"/>
     <row r="129" ht="17.25" customHeight="1"/>
     <row r="130" ht="17.25" customHeight="1"/>
@@ -3936,6 +3952,7 @@
     <row r="997" ht="17.25" customHeight="1"/>
     <row r="998" ht="17.25" customHeight="1"/>
     <row r="999" ht="17.25" customHeight="1"/>
+    <row r="1000" ht="17.25" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="1" orientation="landscape"/>

</xml_diff>